<commit_message>
chore(seed): atualizar catalogo (depositos e itens)
</commit_message>
<xml_diff>
--- a/assets/Tabelas de referência/Depósitos.xlsx
+++ b/assets/Tabelas de referência/Depósitos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5aa5356bde13b7c5/Área de Trabalho/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\TransferToolMobile\TransferTool Mobile\assets\Tabelas de referência\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="8_{68C37976-29BB-4454-9B49-4B31C616ABE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{177C9FA1-1ED4-4E6E-B2B5-82E777905D73}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BFC6940-5867-4FA6-AEF0-EAE5D880959B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,26 +16,14 @@
     <sheet name="Report" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="__bookmark_1">Report!$A$2:$H$69</definedName>
+    <definedName name="__bookmark_1">Report!$A$2:$H$68</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="73">
-  <si>
-    <t>NUTRIÇÃO ALMOXARIFADO ESCOLAS - SMED</t>
-  </si>
-  <si>
-    <t>DEPÓSITO DE UNIFORMES - SMED</t>
-  </si>
-  <si>
-    <t>DEPÓSITO DE MATERIAIS DE MANUTENÇÃO - SMED</t>
-  </si>
-  <si>
-    <t>DEPÓSITO DE MATERIAIS ESCOLARES - SMED</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="72">
   <si>
     <t>ALMOXARIFADO SMED</t>
   </si>
@@ -43,192 +31,9 @@
     <t>DEPÓSITO UTENSÍLIOS NUTRIÇÃO</t>
   </si>
   <si>
-    <t>ALMOXARIFADO EMEF PODALÍRIO INÁCIO DE BARCELLOS</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO EMEI PROFESSORA CLOTILDE SOUZA DO NASCIMENTO</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO PEDACINHO DO CÉU</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO EMEI PEDRO ANTÔNIO PEREIRA DE GODOY</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO EMEF ALCIDES MAIA</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO EMEF ALFREDO JOSÉ JUSTO</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO EMEF ALMIRA FEIJÓ</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO EMEF NOVA PETRÓPOLIS</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO EMEF CECÍLIA MEIRELLES</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO EMEF PAULO FREIRE</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO EMEF EMÍLIA DE OLIVEIRA</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO EMEF CAPITÃO GENTIL MACHADO DE GODOY</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO EMEF CORONEL APARÍCIO GONÇALVES BORGES</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO EMEF CORONEL JOÃO CARLOS VILAGRAN CABRITA</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO EMEF DOM PEDRO II</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO EMEF DUQUE DE CAXIAS</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO EMEF ELISARDO DUARTE NETO</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO EMEF FREDERICO DIHL</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO EMEF HILÁRIO FEIJÓ</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO EMEF IDALINA DE FREITAS LIMA</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO EMEF LEONEL DE MOURA BRIZOLA</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO EMEF MONTEIRO LOBATO</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO EMEF NORMÉLIO PEREIRA DE BARCELLOS</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO EMEF PADRE LÉO SEIDEL</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO EMEF PROFESSORA ALICE DE CARVALHO</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO EMEF PROFESSORA GUILHERMINA DO AMARAL</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO EMEF PROFESSOR JULIANO DO NASCIMENTO</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO EMEF RUI BARBOSA</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO EMEF VEREADOR CLÉO DOS SANTOS</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO EMEF VEREADOR VAGUENIR MANOEL DE FRAGA</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO CMEP ADELINO FERREIRA BORBA</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO FLORESTAN FERNANDES ABESS</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO HELLO KIDS</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO AMOR PERFEITO MATRIZ</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO AMOR PERFEITO 2</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO AMOR PERFEITO FILIAL</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO GENTE NOSSA (MATRIZ)</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO GENTE NOSSA (FILIAL)</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO ÁGAPE</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO LIGA ELEMENTAR DA MULHER</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO AMIGOS DO TAIMBÉ</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO RENATO BATALHA</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO EMEI GLASFIRA</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO RECANTO DA CRIANÇA ESPERANÇA 1</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO RECANTO DA CRIANÇA ESPERANÇA FILIAL</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO CRECHE TIA NENINHA II</t>
-  </si>
-  <si>
-    <t>ALMOXAFIRADO CLUBE DOS LEÕEZINHOS</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO TIA NENINHA I</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO CRECHE TURMA DA MÔNICA</t>
-  </si>
-  <si>
-    <t>DEPÓSITO DE MATERIAIS DE EXPEDIENTE - SMED</t>
-  </si>
-  <si>
-    <t>DEPÓSITO DE MATERIAIS DE LIMPEZA - SMED</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO CEMAEE</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO  EMEF ANTÔNIO DE GODOY</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO TRANSPORTE SMED</t>
-  </si>
-  <si>
-    <t>DEPÓSITO DE MATERIAIS ESPORTIVOS - SMED</t>
-  </si>
-  <si>
-    <t>DEPÓSITO SMED/COMPARTILHE</t>
-  </si>
-  <si>
-    <t>Almoxarifado Central de Matrículas</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO DGA SMED</t>
-  </si>
-  <si>
-    <t>ALMOXARIFADO ESCOLA EM TEMPO INTEGRAL (ETI)</t>
-  </si>
-  <si>
     <t>SEDE ADMINISTRATIVA SMED</t>
   </si>
   <si>
-    <t>Hello Kids Matriz</t>
-  </si>
-  <si>
-    <t>Pacto pela afabetização</t>
-  </si>
-  <si>
     <t>Depósito de origem</t>
   </si>
   <si>
@@ -242,6 +47,198 @@
   </si>
   <si>
     <t>Depósito - Descrição</t>
+  </si>
+  <si>
+    <t>NUTRIÇÃO ALMOXARIFADO ESCOLAS</t>
+  </si>
+  <si>
+    <t>DEPÓSITO DE UNIFORMES</t>
+  </si>
+  <si>
+    <t>DEPÓSITO DE MATERIAIS DE MANUTENÇÃO</t>
+  </si>
+  <si>
+    <t>DEPÓSITO DE MATERIAIS ESCOLARES</t>
+  </si>
+  <si>
+    <t>PODALÍRIO INÁCIO DE BARCELLOS</t>
+  </si>
+  <si>
+    <t>PROFESSORA CLOTILDE SOUZA DO NASCIMENTO</t>
+  </si>
+  <si>
+    <t>PEDACINHO DO CÉU</t>
+  </si>
+  <si>
+    <t>PEDRO ANTÔNIO PEREIRA DE GODOY</t>
+  </si>
+  <si>
+    <t>ALCIDES MAIA</t>
+  </si>
+  <si>
+    <t>ALFREDO JOSÉ JUSTO</t>
+  </si>
+  <si>
+    <t>ALMIRA FEIJÓ</t>
+  </si>
+  <si>
+    <t>NOVA PETRÓPOLIS</t>
+  </si>
+  <si>
+    <t>CECÍLIA MEIRELLES</t>
+  </si>
+  <si>
+    <t>PAULO FREIRE</t>
+  </si>
+  <si>
+    <t>EMÍLIA DE OLIVEIRA</t>
+  </si>
+  <si>
+    <t>CAPITÃO GENTIL MACHADO DE GODOY</t>
+  </si>
+  <si>
+    <t>CORONEL APARÍCIO GONÇALVES BORGES</t>
+  </si>
+  <si>
+    <t>CORONEL JOÃO CARLOS VILAGRAN CABRITA</t>
+  </si>
+  <si>
+    <t>DOM PEDRO II</t>
+  </si>
+  <si>
+    <t>DUQUE DE CAXIAS</t>
+  </si>
+  <si>
+    <t>ELISARDO DUARTE NETO</t>
+  </si>
+  <si>
+    <t>FREDERICO DIHL</t>
+  </si>
+  <si>
+    <t>HILÁRIO FEIJÓ</t>
+  </si>
+  <si>
+    <t>IDALINA DE FREITAS LIMA</t>
+  </si>
+  <si>
+    <t>LEONEL DE MOURA BRIZOLA</t>
+  </si>
+  <si>
+    <t>MONTEIRO LOBATO</t>
+  </si>
+  <si>
+    <t>NORMÉLIO PEREIRA DE BARCELLOS</t>
+  </si>
+  <si>
+    <t>PADRE LÉO SEIDEL</t>
+  </si>
+  <si>
+    <t>PROFESSORA ALICE DE CARVALHO</t>
+  </si>
+  <si>
+    <t>PROFESSORA GUILHERMINA DO AMARAL</t>
+  </si>
+  <si>
+    <t>PROFESSOR JULIANO DO NASCIMENTO</t>
+  </si>
+  <si>
+    <t>RUI BARBOSA</t>
+  </si>
+  <si>
+    <t>VEREADOR CLÉO DOS SANTOS</t>
+  </si>
+  <si>
+    <t>VEREADOR VAGUENIR MANOEL DE FRAGA</t>
+  </si>
+  <si>
+    <t>ADELINO FERREIRA BORBA</t>
+  </si>
+  <si>
+    <t>FLORESTAN FERNANDES ABESS</t>
+  </si>
+  <si>
+    <t>HELLO KIDS FILIAL</t>
+  </si>
+  <si>
+    <t>AMOR PERFEITO MATRIZ</t>
+  </si>
+  <si>
+    <t>AMOR PERFEITO FILIAL</t>
+  </si>
+  <si>
+    <t>GENTE NOSSA MATRIZ</t>
+  </si>
+  <si>
+    <t>GENTE NOSSA FILIAL</t>
+  </si>
+  <si>
+    <t>ÁGAPE</t>
+  </si>
+  <si>
+    <t>LIGA ELEMENTAR DA MULHER</t>
+  </si>
+  <si>
+    <t>AMIGOS DO TAIMBÉ</t>
+  </si>
+  <si>
+    <t>RENATO BATALHA</t>
+  </si>
+  <si>
+    <t>GLASFIRA</t>
+  </si>
+  <si>
+    <t>RECANTO DA CRIANÇA ESPERANÇA MATRIZ</t>
+  </si>
+  <si>
+    <t>RECANTO DA CRIANÇA ESPERANÇA FILIAL</t>
+  </si>
+  <si>
+    <t>TIA NENINHA II</t>
+  </si>
+  <si>
+    <t>CLUBE DOS LEÕEZINHOS</t>
+  </si>
+  <si>
+    <t>TIA NENINHA I</t>
+  </si>
+  <si>
+    <t>TURMA DA MÔNICA</t>
+  </si>
+  <si>
+    <t>MATERIAIS DE EXPEDIENTE</t>
+  </si>
+  <si>
+    <t>MATERIAIS DE LIMPEZA</t>
+  </si>
+  <si>
+    <t>CEMAEE</t>
+  </si>
+  <si>
+    <t>ANTÔNIO DE GODOY</t>
+  </si>
+  <si>
+    <t>TRANSPORTE SMED</t>
+  </si>
+  <si>
+    <t>MATERIAIS ESPORTIVOS</t>
+  </si>
+  <si>
+    <t>COMPARTILHE</t>
+  </si>
+  <si>
+    <t>CENTRAL DE MATRÍCULAS</t>
+  </si>
+  <si>
+    <t>DGA</t>
+  </si>
+  <si>
+    <t>ETI - ESCOLA EM TEMPO INTEGRAL</t>
+  </si>
+  <si>
+    <t>HELLO KIDS MATRIZ</t>
+  </si>
+  <si>
+    <t>PACTO PELA ALFABETIZAÇÃO</t>
   </si>
 </sst>
 </file>
@@ -375,8 +372,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9055C15B-1EDE-4D5F-9E83-45E2F391F45E}" name="Tabela1" displayName="Tabela1" ref="A1:C69" totalsRowShown="0">
-  <autoFilter ref="A1:C69" xr:uid="{9055C15B-1EDE-4D5F-9E83-45E2F391F45E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9055C15B-1EDE-4D5F-9E83-45E2F391F45E}" name="Tabela1" displayName="Tabela1" ref="A1:C68" totalsRowShown="0">
+  <autoFilter ref="A1:C68" xr:uid="{9055C15B-1EDE-4D5F-9E83-45E2F391F45E}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{E057BAF6-C3FA-49F3-895C-FA35C78F2ACD}" name="Depósito - Código" dataDxfId="2"/>
     <tableColumn id="2" xr3:uid="{1A982988-187B-4E31-8F8C-78344E1CC308}" name="Depósito - Descrição" dataDxfId="1"/>
@@ -683,7 +680,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7AC35751-109A-40AE-8756-0C8B52ADD186}">
-  <dimension ref="A1:H69"/>
+  <dimension ref="A1:H68"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
@@ -698,13 +695,13 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>71</v>
+        <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>72</v>
+        <v>7</v>
       </c>
       <c r="C1" t="s">
-        <v>70</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -712,10 +709,10 @@
         <v>10</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>68</v>
+        <v>3</v>
       </c>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
@@ -728,10 +725,10 @@
         <v>44</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>68</v>
+        <v>3</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
@@ -744,10 +741,10 @@
         <v>47</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>68</v>
+        <v>3</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
@@ -760,10 +757,10 @@
         <v>48</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>3</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>68</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
@@ -776,10 +773,10 @@
         <v>49</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>68</v>
+        <v>3</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -792,10 +789,10 @@
         <v>69</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>68</v>
+        <v>3</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
@@ -808,10 +805,10 @@
         <v>70</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
@@ -824,10 +821,10 @@
         <v>71</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
@@ -840,10 +837,10 @@
         <v>72</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
@@ -856,10 +853,10 @@
         <v>73</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
@@ -872,10 +869,10 @@
         <v>74</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
@@ -888,10 +885,10 @@
         <v>75</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
@@ -904,10 +901,10 @@
         <v>76</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
@@ -920,10 +917,10 @@
         <v>77</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
@@ -936,10 +933,10 @@
         <v>78</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
@@ -952,10 +949,10 @@
         <v>79</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
@@ -968,10 +965,10 @@
         <v>80</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
@@ -984,10 +981,10 @@
         <v>81</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
@@ -1000,10 +997,10 @@
         <v>82</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
@@ -1016,10 +1013,10 @@
         <v>83</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
@@ -1032,10 +1029,10 @@
         <v>84</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
@@ -1048,10 +1045,10 @@
         <v>85</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
@@ -1064,10 +1061,10 @@
         <v>86</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
@@ -1080,10 +1077,10 @@
         <v>87</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
@@ -1096,10 +1093,10 @@
         <v>88</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
@@ -1112,10 +1109,10 @@
         <v>89</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D27" s="2"/>
       <c r="E27" s="2"/>
@@ -1128,10 +1125,10 @@
         <v>90</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
@@ -1144,10 +1141,10 @@
         <v>91</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
@@ -1160,10 +1157,10 @@
         <v>92</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
@@ -1176,10 +1173,10 @@
         <v>93</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D31" s="2"/>
       <c r="E31" s="2"/>
@@ -1192,10 +1189,10 @@
         <v>94</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D32" s="2"/>
       <c r="E32" s="2"/>
@@ -1208,10 +1205,10 @@
         <v>95</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D33" s="2"/>
       <c r="E33" s="2"/>
@@ -1224,10 +1221,10 @@
         <v>96</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D34" s="2"/>
       <c r="E34" s="2"/>
@@ -1240,10 +1237,10 @@
         <v>97</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D35" s="2"/>
       <c r="E35" s="2"/>
@@ -1256,10 +1253,10 @@
         <v>98</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D36" s="2"/>
       <c r="E36" s="2"/>
@@ -1272,10 +1269,10 @@
         <v>99</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D37" s="2"/>
       <c r="E37" s="2"/>
@@ -1288,10 +1285,10 @@
         <v>100</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D38" s="2"/>
       <c r="E38" s="2"/>
@@ -1304,10 +1301,10 @@
         <v>103</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D39" s="2"/>
       <c r="E39" s="2"/>
@@ -1320,10 +1317,10 @@
         <v>105</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D40" s="2"/>
       <c r="E40" s="2"/>
@@ -1336,10 +1333,10 @@
         <v>106</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D41" s="2"/>
       <c r="E41" s="2"/>
@@ -1349,13 +1346,13 @@
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D42" s="2"/>
       <c r="E42" s="2"/>
@@ -1365,13 +1362,13 @@
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D43" s="2"/>
       <c r="E43" s="2"/>
@@ -1381,13 +1378,13 @@
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D44" s="2"/>
       <c r="E44" s="2"/>
@@ -1397,13 +1394,13 @@
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D45" s="2"/>
       <c r="E45" s="2"/>
@@ -1413,13 +1410,13 @@
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D46" s="2"/>
       <c r="E46" s="2"/>
@@ -1429,13 +1426,13 @@
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D47" s="2"/>
       <c r="E47" s="2"/>
@@ -1445,13 +1442,13 @@
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D48" s="2"/>
       <c r="E48" s="2"/>
@@ -1461,13 +1458,13 @@
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D49" s="2"/>
       <c r="E49" s="2"/>
@@ -1477,13 +1474,13 @@
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D50" s="2"/>
       <c r="E50" s="2"/>
@@ -1493,13 +1490,13 @@
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D51" s="2"/>
       <c r="E51" s="2"/>
@@ -1509,13 +1506,13 @@
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D52" s="2"/>
       <c r="E52" s="2"/>
@@ -1525,13 +1522,13 @@
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D53" s="2"/>
       <c r="E53" s="2"/>
@@ -1541,13 +1538,13 @@
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D54" s="2"/>
       <c r="E54" s="2"/>
@@ -1557,13 +1554,13 @@
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D55" s="2"/>
       <c r="E55" s="2"/>
@@ -1573,13 +1570,13 @@
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>69</v>
+        <v>3</v>
       </c>
       <c r="D56" s="2"/>
       <c r="E56" s="2"/>
@@ -1589,13 +1586,13 @@
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>68</v>
+        <v>3</v>
       </c>
       <c r="D57" s="2"/>
       <c r="E57" s="2"/>
@@ -1605,13 +1602,13 @@
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>68</v>
+        <v>4</v>
       </c>
       <c r="D58" s="2"/>
       <c r="E58" s="2"/>
@@ -1621,13 +1618,13 @@
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D59" s="2"/>
       <c r="E59" s="2"/>
@@ -1637,13 +1634,13 @@
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D60" s="2"/>
       <c r="E60" s="2"/>
@@ -1653,13 +1650,13 @@
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>69</v>
+        <v>3</v>
       </c>
       <c r="D61" s="2"/>
       <c r="E61" s="2"/>
@@ -1669,13 +1666,13 @@
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>68</v>
+        <v>4</v>
       </c>
       <c r="D62" s="2"/>
       <c r="E62" s="2"/>
@@ -1685,13 +1682,13 @@
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D63" s="2"/>
       <c r="E63" s="2"/>
@@ -1701,13 +1698,13 @@
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D64" s="2"/>
       <c r="E64" s="2"/>
@@ -1717,13 +1714,13 @@
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D65" s="2"/>
       <c r="E65" s="2"/>
@@ -1733,13 +1730,13 @@
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>64</v>
+        <v>2</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D66" s="2"/>
       <c r="E66" s="2"/>
@@ -1749,13 +1746,13 @@
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
-        <v>140</v>
+        <v>188</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D67" s="2"/>
       <c r="E67" s="2"/>
@@ -1765,35 +1762,19 @@
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
-        <v>188</v>
+        <v>217</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>69</v>
+        <v>3</v>
       </c>
       <c r="D68" s="2"/>
       <c r="E68" s="2"/>
       <c r="F68" s="2"/>
       <c r="G68" s="2"/>
       <c r="H68" s="2"/>
-    </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A69" s="1">
-        <v>217</v>
-      </c>
-      <c r="B69" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="C69" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="D69" s="2"/>
-      <c r="E69" s="2"/>
-      <c r="F69" s="2"/>
-      <c r="G69" s="2"/>
-      <c r="H69" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.39369446000000002" right="0.39369446000000002" top="0.27558333000000002" bottom="7.8736109999999998E-2" header="0.5" footer="0.5"/>

</xml_diff>